<commit_message>
chore: rebrand cleanup - all names to Marveile
</commit_message>
<xml_diff>
--- a/data/marveile-katalog-audit.xlsx
+++ b/data/marveile-katalog-audit.xlsx
@@ -1213,7 +1213,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1259,7 +1259,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1305,7 +1305,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1351,7 +1351,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1443,7 +1443,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1489,7 +1489,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1535,7 +1535,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1581,7 +1581,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1627,7 +1627,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1673,7 +1673,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1719,7 +1719,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1765,7 +1765,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1811,7 +1811,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1857,7 +1857,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1903,7 +1903,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1949,7 +1949,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1995,7 +1995,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2041,7 +2041,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2133,7 +2133,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2179,7 +2179,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2225,7 +2225,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2271,7 +2271,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2317,7 +2317,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2363,7 +2363,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2409,7 +2409,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2455,7 +2455,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2501,7 +2501,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2547,7 +2547,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2593,7 +2593,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2639,7 +2639,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2685,7 +2685,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2731,7 +2731,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2823,7 +2823,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>nigoo-legacy</t>
+          <t>marveile-legacy</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>nigoo-legacy:199900</t>
+          <t>marveile-legacy:199900</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>nigoo-legacy:189900</t>
+          <t>marveile-legacy:189900</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>nigoo-legacy:229900</t>
+          <t>marveile-legacy:229900</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>nigoo-legacy:179900</t>
+          <t>marveile-legacy:179900</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>nigoo-legacy:229900</t>
+          <t>marveile-legacy:229900</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>nigoo-legacy:179900</t>
+          <t>marveile-legacy:179900</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -3070,7 +3070,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>nigoo-legacy:179900</t>
+          <t>marveile-legacy:179900</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>nigoo-legacy:219900</t>
+          <t>marveile-legacy:219900</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>nigoo-legacy:149900</t>
+          <t>marveile-legacy:149900</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -3130,7 +3130,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>nigoo-legacy:149900</t>
+          <t>marveile-legacy:149900</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>nigoo-legacy:229900</t>
+          <t>marveile-legacy:229900</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>nigoo-legacy:179900</t>
+          <t>marveile-legacy:179900</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>nigoo-legacy:129900</t>
+          <t>marveile-legacy:129900</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>nigoo-legacy:199900</t>
+          <t>marveile-legacy:199900</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>nigoo-legacy:179900</t>
+          <t>marveile-legacy:179900</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>nigoo-legacy:139900</t>
+          <t>marveile-legacy:139900</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>nigoo-legacy:219900</t>
+          <t>marveile-legacy:219900</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>nigoo-legacy:199900</t>
+          <t>marveile-legacy:199900</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3390,7 +3390,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>nigoo-legacy:204900</t>
+          <t>marveile-legacy:204900</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>nigoo-legacy:239900</t>
+          <t>marveile-legacy:239900</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>nigoo-legacy:159900</t>
+          <t>marveile-legacy:159900</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>nigoo-legacy:190900</t>
+          <t>marveile-legacy:190900</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>nigoo-legacy:199900</t>
+          <t>marveile-legacy:199900</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>nigoo-legacy:149900</t>
+          <t>marveile-legacy:149900</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -3510,7 +3510,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>nigoo-legacy:229900</t>
+          <t>marveile-legacy:229900</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>nigoo-legacy:199900</t>
+          <t>marveile-legacy:199900</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>nigoo-legacy:179900</t>
+          <t>marveile-legacy:179900</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>nigoo-legacy:199900</t>
+          <t>marveile-legacy:199900</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>nigoo-legacy:219900</t>
+          <t>marveile-legacy:219900</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>nigoo-legacy:149900</t>
+          <t>marveile-legacy:149900</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>nigoo-legacy:189900</t>
+          <t>marveile-legacy:189900</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>nigoo-legacy:199900</t>
+          <t>marveile-legacy:199900</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>nigoo-legacy:389900</t>
+          <t>marveile-legacy:389900</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -3730,7 +3730,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>nigoo-legacy:199900</t>
+          <t>marveile-legacy:199900</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>nigoo-legacy:179900</t>
+          <t>marveile-legacy:179900</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>nigoo-legacy:219900</t>
+          <t>marveile-legacy:219900</t>
         </is>
       </c>
       <c r="C45" t="n">

</xml_diff>